<commit_message>
pipeline updated and model code bug fixes
</commit_message>
<xml_diff>
--- a/.Results/Results_With_Sentiment_H1.xlsx
+++ b/.Results/Results_With_Sentiment_H1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
   <si>
     <t>Scenario</t>
   </si>
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -459,6 +459,84 @@
         <v>2.309027494386186</v>
       </c>
     </row>
+    <row r="3" spans="1:8">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3">
+        <v>0.05089006128917312</v>
+      </c>
+      <c r="F3">
+        <v>1.52524081153796</v>
+      </c>
+      <c r="G3">
+        <v>11.66310935539531</v>
+      </c>
+      <c r="H3">
+        <v>2.309027494386186</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4">
+        <v>0.05668224566087705</v>
+      </c>
+      <c r="F4">
+        <v>1.76619364119042</v>
+      </c>
+      <c r="G4">
+        <v>7.993801860147943</v>
+      </c>
+      <c r="H4">
+        <v>2.097449351963747</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5">
+        <v>0.05668224566087705</v>
+      </c>
+      <c r="F5">
+        <v>1.76619364119042</v>
+      </c>
+      <c r="G5">
+        <v>7.993801860147943</v>
+      </c>
+      <c r="H5">
+        <v>2.097449351963747</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
dagsbub resuming and dataset upload to kaggle bug is fixed
</commit_message>
<xml_diff>
--- a/.Results/Results_With_Sentiment_H1.xlsx
+++ b/.Results/Results_With_Sentiment_H1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="37">
   <si>
     <t>Scenario</t>
   </si>
@@ -40,6 +40,18 @@
     <t>Real MAE</t>
   </si>
   <si>
+    <t>Uncertainty</t>
+  </si>
+  <si>
+    <t>PICP</t>
+  </si>
+  <si>
+    <t>Param_Count</t>
+  </si>
+  <si>
+    <t>Best Params</t>
+  </si>
+  <si>
     <t>With Sentiment</t>
   </si>
   <si>
@@ -47,6 +59,72 @@
   </si>
   <si>
     <t>Naive</t>
+  </si>
+  <si>
+    <t>Informer_Base</t>
+  </si>
+  <si>
+    <t>Informer_Base_TTA</t>
+  </si>
+  <si>
+    <t>Informer_DRO</t>
+  </si>
+  <si>
+    <t>Informer_SANorm</t>
+  </si>
+  <si>
+    <t>Informer_FANorm</t>
+  </si>
+  <si>
+    <t>Informer_FANorm_TTA</t>
+  </si>
+  <si>
+    <t>Informer_NoTemporal</t>
+  </si>
+  <si>
+    <t>Informer_NoPositional</t>
+  </si>
+  <si>
+    <t>Informer_NoBothEmbeds</t>
+  </si>
+  <si>
+    <t>Informer_DecOnly</t>
+  </si>
+  <si>
+    <t>Informer_FullAttn</t>
+  </si>
+  <si>
+    <t>Informer_NoDistil</t>
+  </si>
+  <si>
+    <t>Informer_NoProb_NoDistil</t>
+  </si>
+  <si>
+    <t>wo_Gen_Dec</t>
+  </si>
+  <si>
+    <t>Informer_SANorm_NoTemporal</t>
+  </si>
+  <si>
+    <t>Informer_SANorm_DecOnly</t>
+  </si>
+  <si>
+    <t>Informer_FANorm_NoTemporal</t>
+  </si>
+  <si>
+    <t>Informer_FANorm_DecOnly</t>
+  </si>
+  <si>
+    <t>Informer_FANorm_DecOnly_NoTemporal</t>
+  </si>
+  <si>
+    <t>PatchTST_Standalone</t>
+  </si>
+  <si>
+    <t>{'lr': 0.0009025699251123849, 'weight_decay': 1.0807652088882249e-06, 'dropout': 0.04247194877500115, 'batch_size': 16, 'd_model': 16, 'neg_w': 2.388173927043171, 'pos_w': 1.1466509598531762, 'vol_high_w': 1.9598448405246944, 'direction_w': 0.9962413100781786}</t>
+  </si>
+  <si>
+    <t>{'lr': 0.000325437232018654, 'weight_decay': 1.2444490517267001e-06, 'dropout': 0.05682420995623168, 'batch_size': 8, 'd_model': 64, 'patch_len': 8, 'neg_w': 2.8925992732471, 'pos_w': 1.5540128536958397, 'vol_high_w': 2.6157779200967166, 'direction_w': 0.8514914142578691}</t>
   </si>
 </sst>
 </file>
@@ -404,10 +482,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -432,19 +510,31 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E2">
         <v>0.05089006128917312</v>
@@ -459,18 +549,18 @@
         <v>2.309027494386186</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E3">
         <v>0.05089006128917312</v>
@@ -485,18 +575,18 @@
         <v>2.309027494386186</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E4">
         <v>0.05668224566087705</v>
@@ -511,18 +601,18 @@
         <v>2.097449351963747</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="E5">
         <v>0.05668224566087705</v>
@@ -535,6 +625,766 @@
       </c>
       <c r="H5">
         <v>2.097449351963747</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>96</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6">
+        <v>155.9596300125122</v>
+      </c>
+      <c r="F6">
+        <v>112.6020193099976</v>
+      </c>
+      <c r="G6">
+        <v>21994.724609375</v>
+      </c>
+      <c r="H6">
+        <v>133.7209014892578</v>
+      </c>
+      <c r="I6">
+        <v>0.007997959852218628</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>25841</v>
+      </c>
+      <c r="L6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
+        <v>96</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7">
+        <v>154.9854159355164</v>
+      </c>
+      <c r="F7">
+        <v>112.1741056442261</v>
+      </c>
+      <c r="G7">
+        <v>21857.33203125</v>
+      </c>
+      <c r="H7">
+        <v>133.2127380371094</v>
+      </c>
+      <c r="I7">
+        <v>0.007270066533237696</v>
+      </c>
+      <c r="J7">
+        <v>0.003021148036253776</v>
+      </c>
+      <c r="K7">
+        <v>25841</v>
+      </c>
+      <c r="L7" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8">
+        <v>96</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8">
+        <v>159.7057700157166</v>
+      </c>
+      <c r="F8">
+        <v>114.2267107963562</v>
+      </c>
+      <c r="G8">
+        <v>22523.037109375</v>
+      </c>
+      <c r="H8">
+        <v>135.6503143310547</v>
+      </c>
+      <c r="I8">
+        <v>0.008882913738489151</v>
+      </c>
+      <c r="J8">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K8">
+        <v>25841</v>
+      </c>
+      <c r="L8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9">
+        <v>96</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9">
+        <v>156.4667582511902</v>
+      </c>
+      <c r="F9">
+        <v>112.7479910850525</v>
+      </c>
+      <c r="G9">
+        <v>22066.2421875</v>
+      </c>
+      <c r="H9">
+        <v>133.8942565917969</v>
+      </c>
+      <c r="I9">
+        <v>0.005417244508862495</v>
+      </c>
+      <c r="J9">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K9">
+        <v>25941</v>
+      </c>
+      <c r="L9" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10">
+        <v>96</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10">
+        <v>158.6016774177551</v>
+      </c>
+      <c r="F10">
+        <v>113.8292789459229</v>
+      </c>
+      <c r="G10">
+        <v>22367.326171875</v>
+      </c>
+      <c r="H10">
+        <v>135.1783599853516</v>
+      </c>
+      <c r="I10">
+        <v>0.008689535781741142</v>
+      </c>
+      <c r="J10">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K10">
+        <v>25858</v>
+      </c>
+      <c r="L10" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <v>96</v>
+      </c>
+      <c r="C11">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11">
+        <v>155.702817440033</v>
+      </c>
+      <c r="F11">
+        <v>112.476909160614</v>
+      </c>
+      <c r="G11">
+        <v>21958.5078125</v>
+      </c>
+      <c r="H11">
+        <v>133.5723419189453</v>
+      </c>
+      <c r="I11">
+        <v>0.009648709557950497</v>
+      </c>
+      <c r="J11">
+        <v>0.003021148036253776</v>
+      </c>
+      <c r="K11">
+        <v>25858</v>
+      </c>
+      <c r="L11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>96</v>
+      </c>
+      <c r="C12">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12">
+        <v>158.5301280021667</v>
+      </c>
+      <c r="F12">
+        <v>113.8199210166931</v>
+      </c>
+      <c r="G12">
+        <v>22357.23828125</v>
+      </c>
+      <c r="H12">
+        <v>135.1672515869141</v>
+      </c>
+      <c r="I12">
+        <v>0.008033919148147106</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>23377</v>
+      </c>
+      <c r="L12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>96</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>22</v>
+      </c>
+      <c r="E13">
+        <v>161.0049366950989</v>
+      </c>
+      <c r="F13">
+        <v>114.7730827331543</v>
+      </c>
+      <c r="G13">
+        <v>22706.251953125</v>
+      </c>
+      <c r="H13">
+        <v>136.2991638183594</v>
+      </c>
+      <c r="I13">
+        <v>0.008999326266348362</v>
+      </c>
+      <c r="J13">
+        <v>0.003021148036253776</v>
+      </c>
+      <c r="K13">
+        <v>25841</v>
+      </c>
+      <c r="L13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
+      <c r="A14" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14">
+        <v>96</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14">
+        <v>164.2743110656738</v>
+      </c>
+      <c r="F14">
+        <v>116.1945939064026</v>
+      </c>
+      <c r="G14">
+        <v>23167.330078125</v>
+      </c>
+      <c r="H14">
+        <v>137.9872894287109</v>
+      </c>
+      <c r="I14">
+        <v>0.008080456405878067</v>
+      </c>
+      <c r="J14">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K14">
+        <v>23377</v>
+      </c>
+      <c r="L14" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
+      <c r="A15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B15">
+        <v>96</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15">
+        <v>158.5104823112488</v>
+      </c>
+      <c r="F15">
+        <v>113.6602163314819</v>
+      </c>
+      <c r="G15">
+        <v>22354.46484375</v>
+      </c>
+      <c r="H15">
+        <v>134.9775695800781</v>
+      </c>
+      <c r="I15">
+        <v>0.005215178243815899</v>
+      </c>
+      <c r="J15">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K15">
+        <v>10017</v>
+      </c>
+      <c r="L15" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16">
+        <v>96</v>
+      </c>
+      <c r="C16">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16">
+        <v>164.6687030792236</v>
+      </c>
+      <c r="F16">
+        <v>116.3766860961914</v>
+      </c>
+      <c r="G16">
+        <v>23222.94921875</v>
+      </c>
+      <c r="H16">
+        <v>138.2035217285156</v>
+      </c>
+      <c r="I16">
+        <v>0.008144383318722248</v>
+      </c>
+      <c r="J16">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K16">
+        <v>25841</v>
+      </c>
+      <c r="L16" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
+      <c r="A17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B17">
+        <v>96</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>26</v>
+      </c>
+      <c r="E17">
+        <v>162.0582103729248</v>
+      </c>
+      <c r="F17">
+        <v>115.2039647102356</v>
+      </c>
+      <c r="G17">
+        <v>22854.794921875</v>
+      </c>
+      <c r="H17">
+        <v>136.8108520507812</v>
+      </c>
+      <c r="I17">
+        <v>0.009810764342546463</v>
+      </c>
+      <c r="J17">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K17">
+        <v>23393</v>
+      </c>
+      <c r="L17" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12">
+      <c r="A18" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18">
+        <v>96</v>
+      </c>
+      <c r="C18">
+        <v>1</v>
+      </c>
+      <c r="D18" t="s">
+        <v>27</v>
+      </c>
+      <c r="E18">
+        <v>155.1964282989502</v>
+      </c>
+      <c r="F18">
+        <v>112.2667670249939</v>
+      </c>
+      <c r="G18">
+        <v>21887.08984375</v>
+      </c>
+      <c r="H18">
+        <v>133.3227691650391</v>
+      </c>
+      <c r="I18">
+        <v>0.0087230009958148</v>
+      </c>
+      <c r="J18">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K18">
+        <v>23393</v>
+      </c>
+      <c r="L18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
+      <c r="A19" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19">
+        <v>96</v>
+      </c>
+      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="D19" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19">
+        <v>158.4744453430176</v>
+      </c>
+      <c r="F19">
+        <v>113.6959671974182</v>
+      </c>
+      <c r="G19">
+        <v>22349.3828125</v>
+      </c>
+      <c r="H19">
+        <v>135.02001953125</v>
+      </c>
+      <c r="I19">
+        <v>0.008257804438471794</v>
+      </c>
+      <c r="J19">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K19">
+        <v>25841</v>
+      </c>
+      <c r="L19" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12">
+      <c r="A20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20">
+        <v>96</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="s">
+        <v>29</v>
+      </c>
+      <c r="E20">
+        <v>158.7462306022644</v>
+      </c>
+      <c r="F20">
+        <v>113.6735558509827</v>
+      </c>
+      <c r="G20">
+        <v>22387.712890625</v>
+      </c>
+      <c r="H20">
+        <v>134.9934234619141</v>
+      </c>
+      <c r="I20">
+        <v>0.004928024020045996</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>23477</v>
+      </c>
+      <c r="L20" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12">
+      <c r="A21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21">
+        <v>96</v>
+      </c>
+      <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="D21" t="s">
+        <v>30</v>
+      </c>
+      <c r="E21">
+        <v>156.34845495224</v>
+      </c>
+      <c r="F21">
+        <v>112.687885761261</v>
+      </c>
+      <c r="G21">
+        <v>22049.55859375</v>
+      </c>
+      <c r="H21">
+        <v>133.8228759765625</v>
+      </c>
+      <c r="I21">
+        <v>0.003330373438075185</v>
+      </c>
+      <c r="J21">
+        <v>0.004531722054380665</v>
+      </c>
+      <c r="K21">
+        <v>10117</v>
+      </c>
+      <c r="L21" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12">
+      <c r="A22" t="s">
+        <v>12</v>
+      </c>
+      <c r="B22">
+        <v>96</v>
+      </c>
+      <c r="C22">
+        <v>1</v>
+      </c>
+      <c r="D22" t="s">
+        <v>31</v>
+      </c>
+      <c r="E22">
+        <v>156.5421342849731</v>
+      </c>
+      <c r="F22">
+        <v>112.8844141960144</v>
+      </c>
+      <c r="G22">
+        <v>22076.87109375</v>
+      </c>
+      <c r="H22">
+        <v>134.0562591552734</v>
+      </c>
+      <c r="I22">
+        <v>0.008296583779156208</v>
+      </c>
+      <c r="J22">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K22">
+        <v>23394</v>
+      </c>
+      <c r="L22" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12">
+      <c r="A23" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23">
+        <v>96</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="s">
+        <v>32</v>
+      </c>
+      <c r="E23">
+        <v>156.5160870552063</v>
+      </c>
+      <c r="F23">
+        <v>112.7872467041016</v>
+      </c>
+      <c r="G23">
+        <v>22073.203125</v>
+      </c>
+      <c r="H23">
+        <v>133.9408874511719</v>
+      </c>
+      <c r="I23">
+        <v>0.005291115026921034</v>
+      </c>
+      <c r="J23">
+        <v>0.003021148036253776</v>
+      </c>
+      <c r="K23">
+        <v>10034</v>
+      </c>
+      <c r="L23" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12">
+      <c r="A24" t="s">
+        <v>12</v>
+      </c>
+      <c r="B24">
+        <v>96</v>
+      </c>
+      <c r="C24">
+        <v>1</v>
+      </c>
+      <c r="D24" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24">
+        <v>157.7549338340759</v>
+      </c>
+      <c r="F24">
+        <v>113.3330345153809</v>
+      </c>
+      <c r="G24">
+        <v>22247.912109375</v>
+      </c>
+      <c r="H24">
+        <v>134.5890350341797</v>
+      </c>
+      <c r="I24">
+        <v>0.005204910878092051</v>
+      </c>
+      <c r="J24">
+        <v>0.001510574018126888</v>
+      </c>
+      <c r="K24">
+        <v>7570</v>
+      </c>
+      <c r="L24" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
+      <c r="A25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B25">
+        <v>96</v>
+      </c>
+      <c r="C25">
+        <v>1</v>
+      </c>
+      <c r="D25" t="s">
+        <v>34</v>
+      </c>
+      <c r="E25">
+        <v>154.7800302505493</v>
+      </c>
+      <c r="F25">
+        <v>112.109637260437</v>
+      </c>
+      <c r="G25">
+        <v>21828.369140625</v>
+      </c>
+      <c r="H25">
+        <v>133.1361846923828</v>
+      </c>
+      <c r="I25">
+        <v>0.009379984810948372</v>
+      </c>
+      <c r="J25">
+        <v>0.004531722054380665</v>
+      </c>
+      <c r="K25">
+        <v>152729</v>
+      </c>
+      <c r="L25" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>